<commit_message>
Dọn dữ liệu kế toán, tinh gọn skill và lưu quyết định khách hàng
</commit_message>
<xml_diff>
--- a/src/clients/8339629042-001/2026.Q3/Danh sách hóa đơn.xlsx
+++ b/src/clients/8339629042-001/2026.Q3/Danh sách hóa đơn.xlsx
@@ -1,11 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29127"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E8ADA25-2FDE-4F71-BE59-EB722706DA00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet sheetId="1" name="Inv" state="visible" r:id="rId4"/>
+    <sheet name="Inv" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Inv!$A$1:$P$49</definedName>
+  </definedNames>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
@@ -115,7 +122,7 @@
     <t>20/07/2026</t>
   </si>
   <si>
-    <t xml:space="preserve">Huyết thanh làm mờ nếp nhăn THERAMID CLINICAL VITAMIN A 30ml (Hàng biếu tặng không thu tiền)
+    <t>Huyết thanh làm mờ nếp nhăn THERAMID CLINICAL VITAMIN A 30ml (Hàng biếu tặng không thu tiền)
 Huyết thanh dưỡng da TRANSPARENT LAB OIL PATROL SERUM 30ml (Hàng biếu tặng không thu tiền)
 Kem chống nắng TRANSPARENT LAB LIGHTWEIGHT SUNSCREEN SPF50+ 100ml (Hàng biếu tặng không thu tiền) HĐ số 421</t>
   </si>
@@ -180,7 +187,7 @@
     <t>CÔNG TY TNHH THƯƠNG MẠI DỊCH VỤ PHƯƠNG PHÁT</t>
   </si>
   <si>
-    <t xml:space="preserve">3666057272769/ Kem Dưỡng Da Clarins Extra-Firming [Collage] Day Cream Ast 50Ml
+    <t>3666057272769/ Kem Dưỡng Da Clarins Extra-Firming [Collage] Day Cream Ast 50Ml
 3666057272721/ Kem Dưỡng Da Clarins Extra-Firming [Collage] Night Cream Ast 50Ml
 Xuất quảng cáo sản phẩm qua KOL theo hợp đồng số KOC/17082026/CLR/TL ký ngày 17/08/2026, hàng mẫu không thu tiền. HĐ số 188</t>
   </si>
@@ -515,14 +522,17 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="41" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
+  </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -545,8 +555,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -885,9 +896,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:P49"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="10" max="10" width="74.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="14" width="9.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11.5703125" style="1" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
@@ -920,19 +937,19 @@
       <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
       <c r="P1" t="s">
@@ -970,19 +987,19 @@
       <c r="J2" t="s">
         <v>23</v>
       </c>
-      <c r="K2">
+      <c r="K2" s="1">
         <v>99000</v>
       </c>
-      <c r="L2">
-        <v>0</v>
-      </c>
-      <c r="M2">
-        <v>0</v>
-      </c>
-      <c r="N2">
-        <v>0</v>
-      </c>
-      <c r="O2">
+      <c r="L2" s="1">
+        <v>0</v>
+      </c>
+      <c r="M2" s="1">
+        <v>0</v>
+      </c>
+      <c r="N2" s="1">
+        <v>0</v>
+      </c>
+      <c r="O2" s="1">
         <v>99000</v>
       </c>
       <c r="P2" t="s">
@@ -1020,19 +1037,19 @@
       <c r="J3" t="s">
         <v>28</v>
       </c>
-      <c r="K3">
+      <c r="K3" s="1">
         <v>3000000</v>
       </c>
-      <c r="L3">
-        <v>0</v>
-      </c>
-      <c r="M3">
-        <v>0</v>
-      </c>
-      <c r="N3">
+      <c r="L3" s="1">
+        <v>0</v>
+      </c>
+      <c r="M3" s="1">
+        <v>0</v>
+      </c>
+      <c r="N3" s="1">
         <v>240000</v>
       </c>
-      <c r="O3">
+      <c r="O3" s="1">
         <v>3240000</v>
       </c>
       <c r="P3" t="s">
@@ -1070,19 +1087,19 @@
       <c r="J4" t="s">
         <v>32</v>
       </c>
-      <c r="K4">
+      <c r="K4" s="1">
         <v>606018</v>
       </c>
-      <c r="L4">
-        <v>0</v>
-      </c>
-      <c r="M4">
+      <c r="L4" s="1">
+        <v>0</v>
+      </c>
+      <c r="M4" s="1">
         <v>495834</v>
       </c>
-      <c r="N4">
+      <c r="N4" s="1">
         <v>48482</v>
       </c>
-      <c r="O4">
+      <c r="O4" s="1">
         <v>654500</v>
       </c>
       <c r="P4" t="s">
@@ -1120,19 +1137,19 @@
       <c r="J5" t="s">
         <v>34</v>
       </c>
-      <c r="K5">
+      <c r="K5" s="1">
         <v>4185185</v>
       </c>
-      <c r="L5">
-        <v>0</v>
-      </c>
-      <c r="M5">
-        <v>0</v>
-      </c>
-      <c r="N5">
+      <c r="L5" s="1">
+        <v>0</v>
+      </c>
+      <c r="M5" s="1">
+        <v>0</v>
+      </c>
+      <c r="N5" s="1">
         <v>334815</v>
       </c>
-      <c r="O5">
+      <c r="O5" s="1">
         <v>4520000</v>
       </c>
       <c r="P5" t="s">
@@ -1170,19 +1187,19 @@
       <c r="J6" t="s">
         <v>36</v>
       </c>
-      <c r="K6">
+      <c r="K6" s="1">
         <v>3000000</v>
       </c>
-      <c r="L6">
-        <v>0</v>
-      </c>
-      <c r="M6">
-        <v>0</v>
-      </c>
-      <c r="N6">
+      <c r="L6" s="1">
+        <v>0</v>
+      </c>
+      <c r="M6" s="1">
+        <v>0</v>
+      </c>
+      <c r="N6" s="1">
         <v>240000</v>
       </c>
-      <c r="O6">
+      <c r="O6" s="1">
         <v>3240000</v>
       </c>
       <c r="P6" t="s">
@@ -1220,16 +1237,16 @@
       <c r="J7" t="s">
         <v>42</v>
       </c>
-      <c r="K7">
+      <c r="K7" s="1">
         <v>48986</v>
       </c>
-      <c r="L7">
-        <v>0</v>
-      </c>
-      <c r="N7">
-        <v>0</v>
-      </c>
-      <c r="O7">
+      <c r="L7" s="1">
+        <v>0</v>
+      </c>
+      <c r="N7" s="1">
+        <v>0</v>
+      </c>
+      <c r="O7" s="1">
         <v>48986</v>
       </c>
       <c r="P7" t="s">
@@ -1267,19 +1284,19 @@
       <c r="J8" t="s">
         <v>46</v>
       </c>
-      <c r="K8">
+      <c r="K8" s="1">
         <v>7922467</v>
       </c>
-      <c r="L8">
-        <v>0</v>
-      </c>
-      <c r="M8">
-        <v>0</v>
-      </c>
-      <c r="N8">
+      <c r="L8" s="1">
+        <v>0</v>
+      </c>
+      <c r="M8" s="1">
+        <v>0</v>
+      </c>
+      <c r="N8" s="1">
         <v>633797</v>
       </c>
-      <c r="O8">
+      <c r="O8" s="1">
         <v>8556264</v>
       </c>
       <c r="P8" t="s">
@@ -1317,19 +1334,19 @@
       <c r="J9" t="s">
         <v>48</v>
       </c>
-      <c r="K9">
+      <c r="K9" s="1">
         <v>3000000</v>
       </c>
-      <c r="L9">
-        <v>0</v>
-      </c>
-      <c r="M9">
-        <v>0</v>
-      </c>
-      <c r="N9">
+      <c r="L9" s="1">
+        <v>0</v>
+      </c>
+      <c r="M9" s="1">
+        <v>0</v>
+      </c>
+      <c r="N9" s="1">
         <v>240000</v>
       </c>
-      <c r="O9">
+      <c r="O9" s="1">
         <v>3240000</v>
       </c>
       <c r="P9" t="s">
@@ -1367,19 +1384,19 @@
       <c r="J10" t="s">
         <v>50</v>
       </c>
-      <c r="K10">
+      <c r="K10" s="1">
         <v>5308343</v>
       </c>
-      <c r="L10">
-        <v>0</v>
-      </c>
-      <c r="M10">
-        <v>0</v>
-      </c>
-      <c r="N10">
+      <c r="L10" s="1">
+        <v>0</v>
+      </c>
+      <c r="M10" s="1">
+        <v>0</v>
+      </c>
+      <c r="N10" s="1">
         <v>424667</v>
       </c>
-      <c r="O10">
+      <c r="O10" s="1">
         <v>5733010</v>
       </c>
       <c r="P10" t="s">
@@ -1417,19 +1434,19 @@
       <c r="J11" t="s">
         <v>55</v>
       </c>
-      <c r="K11">
+      <c r="K11" s="1">
         <v>5694445</v>
       </c>
-      <c r="L11">
-        <v>0</v>
-      </c>
-      <c r="M11">
-        <v>0</v>
-      </c>
-      <c r="N11">
+      <c r="L11" s="1">
+        <v>0</v>
+      </c>
+      <c r="M11" s="1">
+        <v>0</v>
+      </c>
+      <c r="N11" s="1">
         <v>455555</v>
       </c>
-      <c r="O11">
+      <c r="O11" s="1">
         <v>6150000</v>
       </c>
       <c r="P11" t="s">
@@ -1467,19 +1484,19 @@
       <c r="J12" t="s">
         <v>61</v>
       </c>
-      <c r="K12">
+      <c r="K12" s="1">
         <v>12222222</v>
       </c>
-      <c r="L12">
+      <c r="L12" s="1">
         <v>122222</v>
       </c>
-      <c r="M12">
-        <v>0</v>
-      </c>
-      <c r="N12">
-        <v>0</v>
-      </c>
-      <c r="O12">
+      <c r="M12" s="1">
+        <v>0</v>
+      </c>
+      <c r="N12" s="1">
+        <v>0</v>
+      </c>
+      <c r="O12" s="1">
         <v>12100000</v>
       </c>
       <c r="P12" t="s">
@@ -1517,19 +1534,19 @@
       <c r="J13" t="s">
         <v>65</v>
       </c>
-      <c r="K13">
+      <c r="K13" s="1">
         <v>22222222</v>
       </c>
-      <c r="L13">
+      <c r="L13" s="1">
         <v>222222</v>
       </c>
-      <c r="M13">
-        <v>0</v>
-      </c>
-      <c r="N13">
-        <v>0</v>
-      </c>
-      <c r="O13">
+      <c r="M13" s="1">
+        <v>0</v>
+      </c>
+      <c r="N13" s="1">
+        <v>0</v>
+      </c>
+      <c r="O13" s="1">
         <v>22000000</v>
       </c>
       <c r="P13" t="s">
@@ -1567,19 +1584,19 @@
       <c r="J14" t="s">
         <v>69</v>
       </c>
-      <c r="K14">
+      <c r="K14" s="1">
         <v>41666667</v>
       </c>
-      <c r="L14">
+      <c r="L14" s="1">
         <v>416667</v>
       </c>
-      <c r="M14">
-        <v>0</v>
-      </c>
-      <c r="N14">
-        <v>0</v>
-      </c>
-      <c r="O14">
+      <c r="M14" s="1">
+        <v>0</v>
+      </c>
+      <c r="N14" s="1">
+        <v>0</v>
+      </c>
+      <c r="O14" s="1">
         <v>41250000</v>
       </c>
       <c r="P14" t="s">
@@ -1617,19 +1634,19 @@
       <c r="J15" t="s">
         <v>71</v>
       </c>
-      <c r="K15">
+      <c r="K15" s="1">
         <v>5814141</v>
       </c>
-      <c r="L15">
+      <c r="L15" s="1">
         <v>58141</v>
       </c>
-      <c r="M15">
-        <v>0</v>
-      </c>
-      <c r="N15">
-        <v>0</v>
-      </c>
-      <c r="O15">
+      <c r="M15" s="1">
+        <v>0</v>
+      </c>
+      <c r="N15" s="1">
+        <v>0</v>
+      </c>
+      <c r="O15" s="1">
         <v>5756000</v>
       </c>
       <c r="P15" t="s">
@@ -1667,19 +1684,19 @@
       <c r="J16" t="s">
         <v>75</v>
       </c>
-      <c r="K16">
+      <c r="K16" s="1">
         <v>20000000</v>
       </c>
-      <c r="L16">
+      <c r="L16" s="1">
         <v>200000</v>
       </c>
-      <c r="M16">
-        <v>0</v>
-      </c>
-      <c r="N16">
-        <v>0</v>
-      </c>
-      <c r="O16">
+      <c r="M16" s="1">
+        <v>0</v>
+      </c>
+      <c r="N16" s="1">
+        <v>0</v>
+      </c>
+      <c r="O16" s="1">
         <v>19800000</v>
       </c>
       <c r="P16" t="s">
@@ -1717,19 +1734,19 @@
       <c r="J17" t="s">
         <v>79</v>
       </c>
-      <c r="K17">
+      <c r="K17" s="1">
         <v>11111111</v>
       </c>
-      <c r="L17">
+      <c r="L17" s="1">
         <v>111111</v>
       </c>
-      <c r="M17">
-        <v>0</v>
-      </c>
-      <c r="N17">
-        <v>0</v>
-      </c>
-      <c r="O17">
+      <c r="M17" s="1">
+        <v>0</v>
+      </c>
+      <c r="N17" s="1">
+        <v>0</v>
+      </c>
+      <c r="O17" s="1">
         <v>11000000</v>
       </c>
       <c r="P17" t="s">
@@ -1767,19 +1784,19 @@
       <c r="J18" t="s">
         <v>82</v>
       </c>
-      <c r="K18">
+      <c r="K18" s="1">
         <v>8888889</v>
       </c>
-      <c r="L18">
+      <c r="L18" s="1">
         <v>88889</v>
       </c>
-      <c r="M18">
-        <v>0</v>
-      </c>
-      <c r="N18">
-        <v>0</v>
-      </c>
-      <c r="O18">
+      <c r="M18" s="1">
+        <v>0</v>
+      </c>
+      <c r="N18" s="1">
+        <v>0</v>
+      </c>
+      <c r="O18" s="1">
         <v>8800000</v>
       </c>
       <c r="P18" t="s">
@@ -1817,19 +1834,19 @@
       <c r="J19" t="s">
         <v>85</v>
       </c>
-      <c r="K19">
+      <c r="K19" s="1">
         <v>11111111</v>
       </c>
-      <c r="L19">
+      <c r="L19" s="1">
         <v>111111</v>
       </c>
-      <c r="M19">
-        <v>0</v>
-      </c>
-      <c r="N19">
-        <v>0</v>
-      </c>
-      <c r="O19">
+      <c r="M19" s="1">
+        <v>0</v>
+      </c>
+      <c r="N19" s="1">
+        <v>0</v>
+      </c>
+      <c r="O19" s="1">
         <v>11000000</v>
       </c>
       <c r="P19" t="s">
@@ -1867,19 +1884,19 @@
       <c r="J20" t="s">
         <v>88</v>
       </c>
-      <c r="K20">
+      <c r="K20" s="1">
         <v>10101010</v>
       </c>
-      <c r="L20">
+      <c r="L20" s="1">
         <v>101010</v>
       </c>
-      <c r="M20">
-        <v>0</v>
-      </c>
-      <c r="N20">
-        <v>0</v>
-      </c>
-      <c r="O20">
+      <c r="M20" s="1">
+        <v>0</v>
+      </c>
+      <c r="N20" s="1">
+        <v>0</v>
+      </c>
+      <c r="O20" s="1">
         <v>10000000</v>
       </c>
       <c r="P20" t="s">
@@ -1914,19 +1931,19 @@
       <c r="J21" t="s">
         <v>91</v>
       </c>
-      <c r="K21">
+      <c r="K21" s="1">
         <v>16666667</v>
       </c>
-      <c r="L21">
+      <c r="L21" s="1">
         <v>166667</v>
       </c>
-      <c r="M21">
-        <v>0</v>
-      </c>
-      <c r="N21">
-        <v>0</v>
-      </c>
-      <c r="O21">
+      <c r="M21" s="1">
+        <v>0</v>
+      </c>
+      <c r="N21" s="1">
+        <v>0</v>
+      </c>
+      <c r="O21" s="1">
         <v>16500000</v>
       </c>
       <c r="P21" t="s">
@@ -1964,19 +1981,19 @@
       <c r="J22" t="s">
         <v>95</v>
       </c>
-      <c r="K22">
+      <c r="K22" s="1">
         <v>11111111</v>
       </c>
-      <c r="L22">
+      <c r="L22" s="1">
         <v>111111</v>
       </c>
-      <c r="M22">
-        <v>0</v>
-      </c>
-      <c r="N22">
-        <v>0</v>
-      </c>
-      <c r="O22">
+      <c r="M22" s="1">
+        <v>0</v>
+      </c>
+      <c r="N22" s="1">
+        <v>0</v>
+      </c>
+      <c r="O22" s="1">
         <v>11000000</v>
       </c>
       <c r="P22" t="s">
@@ -2014,19 +2031,19 @@
       <c r="J23" t="s">
         <v>97</v>
       </c>
-      <c r="K23">
+      <c r="K23" s="1">
         <v>11111111</v>
       </c>
-      <c r="L23">
+      <c r="L23" s="1">
         <v>111111</v>
       </c>
-      <c r="M23">
-        <v>0</v>
-      </c>
-      <c r="N23">
-        <v>0</v>
-      </c>
-      <c r="O23">
+      <c r="M23" s="1">
+        <v>0</v>
+      </c>
+      <c r="N23" s="1">
+        <v>0</v>
+      </c>
+      <c r="O23" s="1">
         <v>11000000</v>
       </c>
       <c r="P23" t="s">
@@ -2064,19 +2081,19 @@
       <c r="J24" t="s">
         <v>100</v>
       </c>
-      <c r="K24">
+      <c r="K24" s="1">
         <v>13333333</v>
       </c>
-      <c r="L24">
+      <c r="L24" s="1">
         <v>133333</v>
       </c>
-      <c r="M24">
-        <v>0</v>
-      </c>
-      <c r="N24">
-        <v>0</v>
-      </c>
-      <c r="O24">
+      <c r="M24" s="1">
+        <v>0</v>
+      </c>
+      <c r="N24" s="1">
+        <v>0</v>
+      </c>
+      <c r="O24" s="1">
         <v>13200000</v>
       </c>
       <c r="P24" t="s">
@@ -2111,19 +2128,19 @@
       <c r="J25" t="s">
         <v>103</v>
       </c>
-      <c r="K25">
+      <c r="K25" s="1">
         <v>3181818</v>
       </c>
-      <c r="L25">
+      <c r="L25" s="1">
         <v>31818</v>
       </c>
-      <c r="M25">
-        <v>0</v>
-      </c>
-      <c r="N25">
-        <v>0</v>
-      </c>
-      <c r="O25">
+      <c r="M25" s="1">
+        <v>0</v>
+      </c>
+      <c r="N25" s="1">
+        <v>0</v>
+      </c>
+      <c r="O25" s="1">
         <v>3150000</v>
       </c>
       <c r="P25" t="s">
@@ -2158,19 +2175,19 @@
       <c r="J26" t="s">
         <v>104</v>
       </c>
-      <c r="K26">
+      <c r="K26" s="1">
         <v>857576</v>
       </c>
-      <c r="L26">
+      <c r="L26" s="1">
         <v>8576</v>
       </c>
-      <c r="M26">
-        <v>0</v>
-      </c>
-      <c r="N26">
-        <v>0</v>
-      </c>
-      <c r="O26">
+      <c r="M26" s="1">
+        <v>0</v>
+      </c>
+      <c r="N26" s="1">
+        <v>0</v>
+      </c>
+      <c r="O26" s="1">
         <v>849000</v>
       </c>
       <c r="P26" t="s">
@@ -2208,19 +2225,19 @@
       <c r="J27" t="s">
         <v>108</v>
       </c>
-      <c r="K27">
+      <c r="K27" s="1">
         <v>16666667</v>
       </c>
-      <c r="L27">
+      <c r="L27" s="1">
         <v>166667</v>
       </c>
-      <c r="M27">
-        <v>0</v>
-      </c>
-      <c r="N27">
-        <v>0</v>
-      </c>
-      <c r="O27">
+      <c r="M27" s="1">
+        <v>0</v>
+      </c>
+      <c r="N27" s="1">
+        <v>0</v>
+      </c>
+      <c r="O27" s="1">
         <v>16500000</v>
       </c>
       <c r="P27" t="s">
@@ -2258,19 +2275,19 @@
       <c r="J28" t="s">
         <v>112</v>
       </c>
-      <c r="K28">
+      <c r="K28" s="1">
         <v>13333333</v>
       </c>
-      <c r="L28">
+      <c r="L28" s="1">
         <v>133333</v>
       </c>
-      <c r="M28">
-        <v>0</v>
-      </c>
-      <c r="N28">
-        <v>0</v>
-      </c>
-      <c r="O28">
+      <c r="M28" s="1">
+        <v>0</v>
+      </c>
+      <c r="N28" s="1">
+        <v>0</v>
+      </c>
+      <c r="O28" s="1">
         <v>13200000</v>
       </c>
       <c r="P28" t="s">
@@ -2308,19 +2325,19 @@
       <c r="J29" t="s">
         <v>116</v>
       </c>
-      <c r="K29">
+      <c r="K29" s="1">
         <v>11111111</v>
       </c>
-      <c r="L29">
+      <c r="L29" s="1">
         <v>111111</v>
       </c>
-      <c r="M29">
-        <v>0</v>
-      </c>
-      <c r="N29">
-        <v>0</v>
-      </c>
-      <c r="O29">
+      <c r="M29" s="1">
+        <v>0</v>
+      </c>
+      <c r="N29" s="1">
+        <v>0</v>
+      </c>
+      <c r="O29" s="1">
         <v>11000000</v>
       </c>
       <c r="P29" t="s">
@@ -2358,19 +2375,19 @@
       <c r="J30" t="s">
         <v>120</v>
       </c>
-      <c r="K30">
+      <c r="K30" s="1">
         <v>13333333</v>
       </c>
-      <c r="L30">
+      <c r="L30" s="1">
         <v>133333</v>
       </c>
-      <c r="M30">
-        <v>0</v>
-      </c>
-      <c r="N30">
-        <v>0</v>
-      </c>
-      <c r="O30">
+      <c r="M30" s="1">
+        <v>0</v>
+      </c>
+      <c r="N30" s="1">
+        <v>0</v>
+      </c>
+      <c r="O30" s="1">
         <v>13200000</v>
       </c>
       <c r="P30" t="s">
@@ -2408,19 +2425,19 @@
       <c r="J31" t="s">
         <v>124</v>
       </c>
-      <c r="K31">
+      <c r="K31" s="1">
         <v>11111111</v>
       </c>
-      <c r="L31">
+      <c r="L31" s="1">
         <v>111111</v>
       </c>
-      <c r="M31">
-        <v>0</v>
-      </c>
-      <c r="N31">
-        <v>0</v>
-      </c>
-      <c r="O31">
+      <c r="M31" s="1">
+        <v>0</v>
+      </c>
+      <c r="N31" s="1">
+        <v>0</v>
+      </c>
+      <c r="O31" s="1">
         <v>11000000</v>
       </c>
       <c r="P31" t="s">
@@ -2458,19 +2475,19 @@
       <c r="J32" t="s">
         <v>128</v>
       </c>
-      <c r="K32">
+      <c r="K32" s="1">
         <v>12222222</v>
       </c>
-      <c r="L32">
+      <c r="L32" s="1">
         <v>122222</v>
       </c>
-      <c r="M32">
-        <v>0</v>
-      </c>
-      <c r="N32">
-        <v>0</v>
-      </c>
-      <c r="O32">
+      <c r="M32" s="1">
+        <v>0</v>
+      </c>
+      <c r="N32" s="1">
+        <v>0</v>
+      </c>
+      <c r="O32" s="1">
         <v>12100000</v>
       </c>
       <c r="P32" t="s">
@@ -2508,19 +2525,19 @@
       <c r="J33" t="s">
         <v>129</v>
       </c>
-      <c r="K33">
+      <c r="K33" s="1">
         <v>11111111</v>
       </c>
-      <c r="L33">
+      <c r="L33" s="1">
         <v>111111</v>
       </c>
-      <c r="M33">
-        <v>0</v>
-      </c>
-      <c r="N33">
-        <v>0</v>
-      </c>
-      <c r="O33">
+      <c r="M33" s="1">
+        <v>0</v>
+      </c>
+      <c r="N33" s="1">
+        <v>0</v>
+      </c>
+      <c r="O33" s="1">
         <v>11000000</v>
       </c>
       <c r="P33" t="s">
@@ -2558,19 +2575,19 @@
       <c r="J34" t="s">
         <v>132</v>
       </c>
-      <c r="K34">
+      <c r="K34" s="1">
         <v>16666667</v>
       </c>
-      <c r="L34">
+      <c r="L34" s="1">
         <v>166667</v>
       </c>
-      <c r="M34">
-        <v>0</v>
-      </c>
-      <c r="N34">
-        <v>0</v>
-      </c>
-      <c r="O34">
+      <c r="M34" s="1">
+        <v>0</v>
+      </c>
+      <c r="N34" s="1">
+        <v>0</v>
+      </c>
+      <c r="O34" s="1">
         <v>16500000</v>
       </c>
       <c r="P34" t="s">
@@ -2608,19 +2625,19 @@
       <c r="J35" t="s">
         <v>135</v>
       </c>
-      <c r="K35">
+      <c r="K35" s="1">
         <v>14444444</v>
       </c>
-      <c r="L35">
+      <c r="L35" s="1">
         <v>144444</v>
       </c>
-      <c r="M35">
-        <v>0</v>
-      </c>
-      <c r="N35">
-        <v>0</v>
-      </c>
-      <c r="O35">
+      <c r="M35" s="1">
+        <v>0</v>
+      </c>
+      <c r="N35" s="1">
+        <v>0</v>
+      </c>
+      <c r="O35" s="1">
         <v>14300000</v>
       </c>
       <c r="P35" t="s">
@@ -2655,19 +2672,19 @@
       <c r="J36" t="s">
         <v>137</v>
       </c>
-      <c r="K36">
+      <c r="K36" s="1">
         <v>2229356</v>
       </c>
-      <c r="L36">
+      <c r="L36" s="1">
         <v>22294</v>
       </c>
-      <c r="M36">
-        <v>0</v>
-      </c>
-      <c r="N36">
-        <v>0</v>
-      </c>
-      <c r="O36">
+      <c r="M36" s="1">
+        <v>0</v>
+      </c>
+      <c r="N36" s="1">
+        <v>0</v>
+      </c>
+      <c r="O36" s="1">
         <v>2207062</v>
       </c>
       <c r="P36" t="s">
@@ -2705,19 +2722,19 @@
       <c r="J37" t="s">
         <v>138</v>
       </c>
-      <c r="K37">
+      <c r="K37" s="1">
         <v>13333333</v>
       </c>
-      <c r="L37">
+      <c r="L37" s="1">
         <v>133333</v>
       </c>
-      <c r="M37">
-        <v>0</v>
-      </c>
-      <c r="N37">
-        <v>0</v>
-      </c>
-      <c r="O37">
+      <c r="M37" s="1">
+        <v>0</v>
+      </c>
+      <c r="N37" s="1">
+        <v>0</v>
+      </c>
+      <c r="O37" s="1">
         <v>13200000</v>
       </c>
       <c r="P37" t="s">
@@ -2755,19 +2772,19 @@
       <c r="J38" t="s">
         <v>140</v>
       </c>
-      <c r="K38">
+      <c r="K38" s="1">
         <v>12000000</v>
       </c>
-      <c r="L38">
+      <c r="L38" s="1">
         <v>120000</v>
       </c>
-      <c r="M38">
-        <v>0</v>
-      </c>
-      <c r="N38">
-        <v>0</v>
-      </c>
-      <c r="O38">
+      <c r="M38" s="1">
+        <v>0</v>
+      </c>
+      <c r="N38" s="1">
+        <v>0</v>
+      </c>
+      <c r="O38" s="1">
         <v>11880000</v>
       </c>
       <c r="P38" t="s">
@@ -2805,19 +2822,19 @@
       <c r="J39" t="s">
         <v>141</v>
       </c>
-      <c r="K39">
+      <c r="K39" s="1">
         <v>11111111</v>
       </c>
-      <c r="L39">
+      <c r="L39" s="1">
         <v>111111</v>
       </c>
-      <c r="M39">
-        <v>0</v>
-      </c>
-      <c r="N39">
-        <v>0</v>
-      </c>
-      <c r="O39">
+      <c r="M39" s="1">
+        <v>0</v>
+      </c>
+      <c r="N39" s="1">
+        <v>0</v>
+      </c>
+      <c r="O39" s="1">
         <v>11000000</v>
       </c>
       <c r="P39" t="s">
@@ -2855,19 +2872,19 @@
       <c r="J40" t="s">
         <v>142</v>
       </c>
-      <c r="K40">
+      <c r="K40" s="1">
         <v>15555556</v>
       </c>
-      <c r="L40">
+      <c r="L40" s="1">
         <v>155556</v>
       </c>
-      <c r="M40">
-        <v>0</v>
-      </c>
-      <c r="N40">
-        <v>0</v>
-      </c>
-      <c r="O40">
+      <c r="M40" s="1">
+        <v>0</v>
+      </c>
+      <c r="N40" s="1">
+        <v>0</v>
+      </c>
+      <c r="O40" s="1">
         <v>15400000</v>
       </c>
       <c r="P40" t="s">
@@ -2905,19 +2922,19 @@
       <c r="J41" t="s">
         <v>144</v>
       </c>
-      <c r="K41">
+      <c r="K41" s="1">
         <v>1666667</v>
       </c>
-      <c r="L41">
+      <c r="L41" s="1">
         <v>16667</v>
       </c>
-      <c r="M41">
-        <v>0</v>
-      </c>
-      <c r="N41">
-        <v>0</v>
-      </c>
-      <c r="O41">
+      <c r="M41" s="1">
+        <v>0</v>
+      </c>
+      <c r="N41" s="1">
+        <v>0</v>
+      </c>
+      <c r="O41" s="1">
         <v>1650000</v>
       </c>
       <c r="P41" t="s">
@@ -2955,19 +2972,19 @@
       <c r="J42" t="s">
         <v>148</v>
       </c>
-      <c r="K42">
+      <c r="K42" s="1">
         <v>12222222</v>
       </c>
-      <c r="L42">
+      <c r="L42" s="1">
         <v>122222</v>
       </c>
-      <c r="M42">
-        <v>0</v>
-      </c>
-      <c r="N42">
-        <v>0</v>
-      </c>
-      <c r="O42">
+      <c r="M42" s="1">
+        <v>0</v>
+      </c>
+      <c r="N42" s="1">
+        <v>0</v>
+      </c>
+      <c r="O42" s="1">
         <v>12100000</v>
       </c>
       <c r="P42" t="s">
@@ -3005,19 +3022,19 @@
       <c r="J43" t="s">
         <v>150</v>
       </c>
-      <c r="K43">
+      <c r="K43" s="1">
         <v>22222222</v>
       </c>
-      <c r="L43">
+      <c r="L43" s="1">
         <v>222222</v>
       </c>
-      <c r="M43">
-        <v>0</v>
-      </c>
-      <c r="N43">
-        <v>0</v>
-      </c>
-      <c r="O43">
+      <c r="M43" s="1">
+        <v>0</v>
+      </c>
+      <c r="N43" s="1">
+        <v>0</v>
+      </c>
+      <c r="O43" s="1">
         <v>22000000</v>
       </c>
       <c r="P43" t="s">
@@ -3055,19 +3072,19 @@
       <c r="J44" t="s">
         <v>152</v>
       </c>
-      <c r="K44">
+      <c r="K44" s="1">
         <v>11111111</v>
       </c>
-      <c r="L44">
+      <c r="L44" s="1">
         <v>111111</v>
       </c>
-      <c r="M44">
-        <v>0</v>
-      </c>
-      <c r="N44">
-        <v>0</v>
-      </c>
-      <c r="O44">
+      <c r="M44" s="1">
+        <v>0</v>
+      </c>
+      <c r="N44" s="1">
+        <v>0</v>
+      </c>
+      <c r="O44" s="1">
         <v>11000000</v>
       </c>
       <c r="P44" t="s">
@@ -3105,19 +3122,19 @@
       <c r="J45" t="s">
         <v>155</v>
       </c>
-      <c r="K45">
+      <c r="K45" s="1">
         <v>13333333</v>
       </c>
-      <c r="L45">
+      <c r="L45" s="1">
         <v>133333</v>
       </c>
-      <c r="M45">
-        <v>0</v>
-      </c>
-      <c r="N45">
-        <v>0</v>
-      </c>
-      <c r="O45">
+      <c r="M45" s="1">
+        <v>0</v>
+      </c>
+      <c r="N45" s="1">
+        <v>0</v>
+      </c>
+      <c r="O45" s="1">
         <v>13200000</v>
       </c>
       <c r="P45" t="s">
@@ -3155,19 +3172,19 @@
       <c r="J46" t="s">
         <v>159</v>
       </c>
-      <c r="K46">
+      <c r="K46" s="1">
         <v>13333333</v>
       </c>
-      <c r="L46">
+      <c r="L46" s="1">
         <v>133333</v>
       </c>
-      <c r="M46">
-        <v>0</v>
-      </c>
-      <c r="N46">
-        <v>0</v>
-      </c>
-      <c r="O46">
+      <c r="M46" s="1">
+        <v>0</v>
+      </c>
+      <c r="N46" s="1">
+        <v>0</v>
+      </c>
+      <c r="O46" s="1">
         <v>13200000</v>
       </c>
       <c r="P46" t="s">
@@ -3205,19 +3222,19 @@
       <c r="J47" t="s">
         <v>161</v>
       </c>
-      <c r="K47">
+      <c r="K47" s="1">
         <v>13333333</v>
       </c>
-      <c r="L47">
+      <c r="L47" s="1">
         <v>133333</v>
       </c>
-      <c r="M47">
-        <v>0</v>
-      </c>
-      <c r="N47">
-        <v>0</v>
-      </c>
-      <c r="O47">
+      <c r="M47" s="1">
+        <v>0</v>
+      </c>
+      <c r="N47" s="1">
+        <v>0</v>
+      </c>
+      <c r="O47" s="1">
         <v>13200000</v>
       </c>
       <c r="P47" t="s">
@@ -3255,19 +3272,19 @@
       <c r="J48" t="s">
         <v>163</v>
       </c>
-      <c r="K48">
+      <c r="K48" s="1">
         <v>11111111</v>
       </c>
-      <c r="L48">
+      <c r="L48" s="1">
         <v>111111</v>
       </c>
-      <c r="M48">
-        <v>0</v>
-      </c>
-      <c r="N48">
-        <v>0</v>
-      </c>
-      <c r="O48">
+      <c r="M48" s="1">
+        <v>0</v>
+      </c>
+      <c r="N48" s="1">
+        <v>0</v>
+      </c>
+      <c r="O48" s="1">
         <v>11000000</v>
       </c>
       <c r="P48" t="s">
@@ -3302,19 +3319,19 @@
       <c r="J49" t="s">
         <v>164</v>
       </c>
-      <c r="K49">
+      <c r="K49" s="1">
         <v>2743559</v>
       </c>
-      <c r="L49">
+      <c r="L49" s="1">
         <v>27436</v>
       </c>
-      <c r="M49">
-        <v>0</v>
-      </c>
-      <c r="N49">
-        <v>0</v>
-      </c>
-      <c r="O49">
+      <c r="M49" s="1">
+        <v>0</v>
+      </c>
+      <c r="N49" s="1">
+        <v>0</v>
+      </c>
+      <c r="O49" s="1">
         <v>2716123</v>
       </c>
       <c r="P49" t="s">
@@ -3322,7 +3339,8 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:P49" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>